<commit_message>
Bulk import: step-by-step guide, sample Excel file, reliable xlsx reading
- «ورود دیتابیس برند»: a 5-step guide at the top and «دریافت فایل نمونه (Excel)»
  (GET /admin/brand-imports/sample.xlsx; its titles are recognized automatically)
- Knowledge center: a box explaining that its files are reference only, with
  one-click paths to brand import and Excel import and their sample files
- «قطعات»: «ورود گروهی قطعه» button
- xlsx reading: entries opened by name with our zip reader (sheet list and
  shared strings first, each sheet streamed with backpressure). ExcelJS's
  whole-file streaming sometimes lost entries when a sheet came before the
  shared strings (as Excel saves them): empty cells or a crash
- Test: the sample downloads, every column is recognized, 3 new rows, 0 errors

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/import/sample-import-with-errors.xlsx
+++ b/docs/import/sample-import-with-errors.xlsx
@@ -70,7 +70,7 @@
     <t>is_active</t>
   </si>
   <si>
-    <t>00CJIQT</t>
+    <t>00DTLGD</t>
   </si>
   <si>
     <t>قطعهٔ واردشده آزمایشی</t>
@@ -106,28 +106,28 @@
     <t>کد عددی</t>
   </si>
   <si>
-    <t>CUR-MVDCJIQT</t>
+    <t>CUR-MVDDTLGD</t>
   </si>
   <si>
     <t>TOMAN</t>
   </si>
   <si>
-    <t>QTY-MVDCJIQT</t>
-  </si>
-  <si>
-    <t>NEG-MVDCJIQT</t>
+    <t>QTY-MVDDTLGD</t>
+  </si>
+  <si>
+    <t>NEG-MVDDTLGD</t>
   </si>
   <si>
     <t>-5</t>
   </si>
   <si>
-    <t>CAT-MVDCJIQT</t>
+    <t>CAT-MVDDTLGD</t>
   </si>
   <si>
     <t>NOPE</t>
   </si>
   <si>
-    <t>FX-MVDCJIQT</t>
+    <t>FX-MVDDTLGD</t>
   </si>
 </sst>
 </file>

</xml_diff>